<commit_message>
Sync balance workbook with runtime drops data
</commit_message>
<xml_diff>
--- a/balance/Spiria_Game_Balance_v1.0.xlsx
+++ b/balance/Spiria_Game_Balance_v1.0.xlsx
@@ -2540,7 +2540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2974,7 +2974,7 @@
         </is>
       </c>
       <c r="C12" s="63" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="D12" s="20" t="inlineStr">
         <is>
@@ -3003,44 +3003,42 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
-        <is>
-          <t>Map1</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="inlineStr">
-        <is>
-          <t>region_id</t>
-        </is>
-      </c>
-      <c r="C13" s="63" t="inlineStr">
-        <is>
-          <t>starlight_forest</t>
-        </is>
-      </c>
-      <c r="D13" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E13" s="20" t="inlineStr">
-        <is>
-          <t>현재 적용 지역 ID</t>
-        </is>
-      </c>
-      <c r="F13" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H13" s="20" t="inlineStr">
-        <is>
-          <t>src/data/regions.ts</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>mana_single_drop_chance_per_expedition</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>탐험 1회당 마나 단일 드랍 확률</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>마나 획득 빈도 증가</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>마나 획득 빈도 감소</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>src/data/drops.ts</t>
         </is>
       </c>
     </row>
@@ -3052,12 +3050,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>region_name</t>
+          <t>region_id</t>
         </is>
       </c>
       <c r="C14" s="63" t="inlineStr">
         <is>
-          <t>별빛 숲속</t>
+          <t>starlight_forest</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -3067,7 +3065,7 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>현재 적용 지역명</t>
+          <t>현재 적용 지역 ID</t>
         </is>
       </c>
       <c r="F14" s="20" t="inlineStr">
@@ -3094,30 +3092,32 @@
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>unlock_level</t>
-        </is>
-      </c>
-      <c r="C15" s="63" t="n">
-        <v>1</v>
+          <t>region_name</t>
+        </is>
+      </c>
+      <c r="C15" s="63" t="inlineStr">
+        <is>
+          <t>별빛 숲속</t>
+        </is>
       </c>
       <c r="D15" s="20" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>입장 레벨</t>
+          <t>현재 적용 지역명</t>
         </is>
       </c>
       <c r="F15" s="20" t="inlineStr">
         <is>
-          <t>해금 지연</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G15" s="20" t="inlineStr">
         <is>
-          <t>해금 빨라짐</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H15" s="20" t="inlineStr">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>recommended_level</t>
+          <t>unlock_level</t>
         </is>
       </c>
       <c r="C16" s="63" t="n">
@@ -3147,17 +3147,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>권장 레벨</t>
+          <t>입장 레벨</t>
         </is>
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>권장치 상승</t>
+          <t>해금 지연</t>
         </is>
       </c>
       <c r="G16" s="20" t="inlineStr">
         <is>
-          <t>권장치 하락</t>
+          <t>해금 빨라짐</t>
         </is>
       </c>
       <c r="H16" s="20" t="inlineStr">
@@ -3174,30 +3174,30 @@
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>weight_material</t>
+          <t>recommended_level</t>
         </is>
       </c>
       <c r="C17" s="63" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D17" s="20" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>level</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>탐색률 재료 기여</t>
+          <t>권장 레벨</t>
         </is>
       </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>탐색률 해당 항목 비중↑</t>
+          <t>권장치 상승</t>
         </is>
       </c>
       <c r="G17" s="20" t="inlineStr">
         <is>
-          <t>비중↓</t>
+          <t>권장치 하락</t>
         </is>
       </c>
       <c r="H17" s="20" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>weight_spirit</t>
+          <t>weight_material</t>
         </is>
       </c>
       <c r="C18" s="63" t="n">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>탐색률 정령 기여</t>
+          <t>탐색률 재료 기여</t>
         </is>
       </c>
       <c r="F18" s="20" t="inlineStr">
@@ -3254,7 +3254,7 @@
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>weight_regional</t>
+          <t>weight_spirit</t>
         </is>
       </c>
       <c r="C19" s="63" t="n">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>탐색률 지역 기여</t>
+          <t>탐색률 정령 기여</t>
         </is>
       </c>
       <c r="F19" s="20" t="inlineStr">
@@ -3294,11 +3294,11 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>weight_treasure</t>
+          <t>weight_regional</t>
         </is>
       </c>
       <c r="C20" s="63" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>탐색률 보물 기여</t>
+          <t>탐색률 지역 기여</t>
         </is>
       </c>
       <c r="F20" s="20" t="inlineStr">
@@ -3334,30 +3334,30 @@
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>total_material_discovery</t>
+          <t>weight_treasure</t>
         </is>
       </c>
       <c r="C21" s="63" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D21" s="20" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>weight</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>재료 발견 총량</t>
+          <t>탐색률 보물 기여</t>
         </is>
       </c>
       <c r="F21" s="20" t="inlineStr">
         <is>
-          <t>완료 난이도↑</t>
+          <t>탐색률 해당 항목 비중↑</t>
         </is>
       </c>
       <c r="G21" s="20" t="inlineStr">
         <is>
-          <t>완료 난이도↓</t>
+          <t>비중↓</t>
         </is>
       </c>
       <c r="H21" s="20" t="inlineStr">
@@ -3374,11 +3374,11 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>total_spirit_discovery</t>
+          <t>total_material_discovery</t>
         </is>
       </c>
       <c r="C22" s="63" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>정령 발견 총량</t>
+          <t>재료 발견 총량</t>
         </is>
       </c>
       <c r="F22" s="20" t="inlineStr">
@@ -3414,11 +3414,11 @@
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>total_regional_discovery</t>
+          <t>total_spirit_discovery</t>
         </is>
       </c>
       <c r="C23" s="63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D23" s="20" t="inlineStr">
         <is>
@@ -3427,7 +3427,7 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>지역 발견 총량</t>
+          <t>정령 발견 총량</t>
         </is>
       </c>
       <c r="F23" s="20" t="inlineStr">
@@ -3454,75 +3454,73 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
+          <t>total_regional_discovery</t>
+        </is>
+      </c>
+      <c r="C24" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>지역 발견 총량</t>
+        </is>
+      </c>
+      <c r="F24" s="20" t="inlineStr">
+        <is>
+          <t>완료 난이도↑</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>완료 난이도↓</t>
+        </is>
+      </c>
+      <c r="H24" s="20" t="inlineStr">
+        <is>
+          <t>src/data/regions.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>Map1</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
           <t>total_treasure_discovery</t>
         </is>
       </c>
-      <c r="C24" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="C25" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="E25" s="20" t="inlineStr">
         <is>
           <t>보물 발견 총량</t>
         </is>
       </c>
-      <c r="F24" s="20" t="inlineStr">
+      <c r="F25" s="20" t="inlineStr">
         <is>
           <t>완료 난이도↑</t>
         </is>
       </c>
-      <c r="G24" s="20" t="inlineStr">
+      <c r="G25" s="20" t="inlineStr">
         <is>
           <t>완료 난이도↓</t>
         </is>
       </c>
-      <c r="H24" s="20" t="inlineStr">
-        <is>
-          <t>src/data/regions.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Map2</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>region_id</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>wind_canyon</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>현재 적용 지역 ID</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="20" t="inlineStr">
         <is>
           <t>src/data/regions.ts</t>
         </is>
@@ -3536,12 +3534,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>region_name</t>
+          <t>region_id</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>바람의 협곡</t>
+          <t>wind_canyon</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3551,7 +3549,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>현재 적용 지역명</t>
+          <t>현재 적용 지역 ID</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3578,30 +3576,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>unlock_level</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>10</v>
+          <t>region_name</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>바람의 협곡</t>
+        </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>입장 레벨</t>
+          <t>현재 적용 지역명</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>해금 지연</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>해금 빨라짐</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3618,7 +3618,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>recommended_level</t>
+          <t>unlock_level</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3631,17 +3631,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>권장 레벨</t>
+          <t>입장 레벨</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>권장치 상승</t>
+          <t>해금 지연</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>권장치 하락</t>
+          <t>해금 빨라짐</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3658,30 +3658,30 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>mana_cost</t>
+          <t>recommended_level</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>mana</t>
+          <t>level</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>탐사 1회 입장 소모 마나</t>
+          <t>권장 레벨</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>비용 증가</t>
+          <t>권장치 상승</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>비용 감소</t>
+          <t>권장치 하락</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3698,30 +3698,30 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>explore_steps</t>
+          <t>mana_cost</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>mana</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>탐색 행동 횟수</t>
+          <t>탐사 1회 입장 소모 마나</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>탐험 길어짐</t>
+          <t>비용 증가</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>탐험 짧아짐</t>
+          <t>비용 감소</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3738,32 +3738,30 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>trace_item_id</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>wind_trace</t>
-        </is>
+          <t>explore_steps</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>10</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>지역 흔적 아이템 ID</t>
+          <t>탐색 행동 횟수</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>탐험 길어짐</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>탐험 짧아짐</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3780,12 +3778,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>trace_name</t>
+          <t>trace_item_id</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>바람의 메아리</t>
+          <t>wind_trace</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3795,7 +3793,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>지역 흔적 아이템명</t>
+          <t>지역 흔적 아이템 ID</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3822,30 +3820,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>hidden_stage_required_amount</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>20</v>
+          <t>trace_name</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>바람의 메아리</t>
+        </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Hidden Stage 입장 흔적 수</t>
+          <t>지역 흔적 아이템명</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>입장 난이도↑</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>입장 난이도↓</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3862,32 +3862,30 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>next_region_id</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>frozen_lake</t>
-        </is>
+          <t>hidden_stage_required_amount</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>20</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>다음 지역 ID</t>
+          <t>Hidden Stage 입장 흔적 수</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>입장 난이도↑</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>입장 난이도↓</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3904,30 +3902,32 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>next_region_unlock_level</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>25</v>
+          <t>next_region_id</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>frozen_lake</t>
+        </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>다음 지역 해금 레벨</t>
+          <t>다음 지역 ID</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>해금 지연</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>해금 빨라짐</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3944,30 +3944,30 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>weight_material</t>
+          <t>next_region_unlock_level</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>level</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>탐색률 재료 기여</t>
+          <t>다음 지역 해금 레벨</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>비중↑</t>
+          <t>해금 지연</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>비중↓</t>
+          <t>해금 빨라짐</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>weight_spirit</t>
+          <t>weight_material</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>탐색률 정령 기여</t>
+          <t>탐색률 재료 기여</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>weight_regional</t>
+          <t>weight_spirit</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>탐색률 지역 기여</t>
+          <t>탐색률 정령 기여</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4064,11 +4064,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>weight_treasure</t>
+          <t>weight_regional</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -4077,7 +4077,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>탐색률 보물 기여</t>
+          <t>탐색률 지역 기여</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4104,30 +4104,30 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>total_material_discovery</t>
+          <t>weight_treasure</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>weight</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>재료 발견 총량</t>
+          <t>탐색률 보물 기여</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>완료 난이도↑</t>
+          <t>비중↑</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>완료 난이도↓</t>
+          <t>비중↓</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -4144,11 +4144,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>total_spirit_discovery</t>
+          <t>total_material_discovery</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>정령 발견 총량</t>
+          <t>재료 발견 총량</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4184,11 +4184,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>total_regional_discovery</t>
+          <t>total_spirit_discovery</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>지역 발견 총량</t>
+          <t>정령 발견 총량</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4224,11 +4224,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>total_treasure_discovery</t>
+          <t>total_regional_discovery</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>보물 발견 총량</t>
+          <t>지역 발견 총량</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4259,37 +4259,35 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Map3</t>
+          <t>Map2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>region_id</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>frozen_lake</t>
-        </is>
+          <t>total_treasure_discovery</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>현재 적용 지역 ID</t>
+          <t>보물 발견 총량</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>완료 난이도↑</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>완료 난이도↓</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4306,12 +4304,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>region_name</t>
+          <t>region_id</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>얼어붙은 설원</t>
+          <t>frozen_lake</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4321,7 +4319,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>현재 적용 지역명</t>
+          <t>현재 적용 지역 ID</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4348,30 +4346,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>unlock_level</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>25</v>
+          <t>region_name</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>얼어붙은 설원</t>
+        </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>입장 레벨</t>
+          <t>현재 적용 지역명</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>해금 지연</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>해금 빨라짐</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -4388,7 +4388,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>recommended_level</t>
+          <t>unlock_level</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -4401,17 +4401,17 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>권장 레벨</t>
+          <t>입장 레벨</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>권장치 상승</t>
+          <t>해금 지연</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>권장치 하락</t>
+          <t>해금 빨라짐</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4428,30 +4428,30 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>mana_cost</t>
+          <t>recommended_level</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>mana</t>
+          <t>level</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>탐사 1회 입장 소모 마나</t>
+          <t>권장 레벨</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>비용 증가</t>
+          <t>권장치 상승</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>비용 감소</t>
+          <t>권장치 하락</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4468,30 +4468,30 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>explore_steps</t>
+          <t>mana_cost</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>mana</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>탐색 행동 횟수</t>
+          <t>탐사 1회 입장 소모 마나</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>탐험 길어짐</t>
+          <t>비용 증가</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>탐험 짧아짐</t>
+          <t>비용 감소</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4508,32 +4508,30 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>trace_item_id</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>lake_trace</t>
-        </is>
+          <t>explore_steps</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>10</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>지역 흔적 아이템 ID</t>
+          <t>탐색 행동 횟수</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>탐험 길어짐</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>탐험 짧아짐</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4550,12 +4548,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>trace_name</t>
+          <t>trace_item_id</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>설원의 기억</t>
+          <t>lake_trace</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4565,7 +4563,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>지역 흔적 아이템명</t>
+          <t>지역 흔적 아이템 ID</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4592,30 +4590,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>hidden_stage_required_amount</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>20</v>
+          <t>trace_name</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>설원의 기억</t>
+        </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Hidden Stage 입장 흔적 수</t>
+          <t>지역 흔적 아이템명</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>입장 난이도↑</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>입장 난이도↓</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4632,32 +4632,30 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>next_region_id</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>flame_ruins</t>
-        </is>
+          <t>hidden_stage_required_amount</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>20</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>다음 지역 ID</t>
+          <t>Hidden Stage 입장 흔적 수</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>입장 난이도↑</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>입장 난이도↓</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -4674,30 +4672,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>next_region_unlock_level</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>50</v>
+          <t>next_region_id</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>flame_ruins</t>
+        </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>다음 지역 해금 레벨</t>
+          <t>다음 지역 ID</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>해금 지연</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>해금 빨라짐</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4714,30 +4714,30 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>weight_material</t>
+          <t>next_region_unlock_level</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>level</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>탐색률 재료 기여</t>
+          <t>다음 지역 해금 레벨</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>비중↑</t>
+          <t>해금 지연</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>비중↓</t>
+          <t>해금 빨라짐</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -4754,7 +4754,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>weight_spirit</t>
+          <t>weight_material</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>탐색률 정령 기여</t>
+          <t>탐색률 재료 기여</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4794,7 +4794,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>weight_regional</t>
+          <t>weight_spirit</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -4807,7 +4807,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>탐색률 지역 기여</t>
+          <t>탐색률 정령 기여</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4834,11 +4834,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>weight_treasure</t>
+          <t>weight_regional</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -4847,7 +4847,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>탐색률 보물 기여</t>
+          <t>탐색률 지역 기여</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4874,30 +4874,30 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>total_material_discovery</t>
+          <t>weight_treasure</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>weight</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>재료 발견 총량</t>
+          <t>탐색률 보물 기여</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>완료 난이도↑</t>
+          <t>비중↑</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>완료 난이도↓</t>
+          <t>비중↓</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4914,11 +4914,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>total_spirit_discovery</t>
+          <t>total_material_discovery</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>정령 발견 총량</t>
+          <t>재료 발견 총량</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -4954,11 +4954,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>total_regional_discovery</t>
+          <t>total_spirit_discovery</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -4967,7 +4967,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>지역 발견 총량</t>
+          <t>정령 발견 총량</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -4994,11 +4994,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>total_treasure_discovery</t>
+          <t>total_regional_discovery</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -5007,7 +5007,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>보물 발견 총량</t>
+          <t>지역 발견 총량</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5029,37 +5029,35 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Map4</t>
+          <t>Map3</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>region_id</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>flame_ruins</t>
-        </is>
+          <t>total_treasure_discovery</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>현재 적용 지역 ID</t>
+          <t>보물 발견 총량</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>완료 난이도↑</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>완료 난이도↓</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5076,12 +5074,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>region_name</t>
+          <t>region_id</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>화염의 산맥</t>
+          <t>flame_ruins</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -5091,7 +5089,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>현재 적용 지역명</t>
+          <t>현재 적용 지역 ID</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5118,30 +5116,32 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>unlock_level</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>50</v>
+          <t>region_name</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>화염의 산맥</t>
+        </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>입장 레벨</t>
+          <t>현재 적용 지역명</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>해금 지연</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>해금 빨라짐</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>recommended_level</t>
+          <t>unlock_level</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -5171,17 +5171,17 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>권장 레벨</t>
+          <t>입장 레벨</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>권장치 상승</t>
+          <t>해금 지연</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>권장치 하락</t>
+          <t>해금 빨라짐</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -5198,30 +5198,30 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>mana_cost</t>
+          <t>recommended_level</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>mana</t>
+          <t>level</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>탐사 1회 입장 소모 마나</t>
+          <t>권장 레벨</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>비용 증가</t>
+          <t>권장치 상승</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>비용 감소</t>
+          <t>권장치 하락</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -5238,30 +5238,30 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>explore_steps</t>
+          <t>mana_cost</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>mana</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>탐색 행동 횟수</t>
+          <t>탐사 1회 입장 소모 마나</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>탐험 길어짐</t>
+          <t>비용 증가</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>탐험 짧아짐</t>
+          <t>비용 감소</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -5278,32 +5278,30 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>trace_item_id</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>ruins_trace</t>
-        </is>
+          <t>explore_steps</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>10</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>지역 흔적 아이템 ID</t>
+          <t>탐색 행동 횟수</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>탐험 길어짐</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>탐험 짧아짐</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -5320,12 +5318,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>trace_name</t>
+          <t>trace_item_id</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>화염의 잔재</t>
+          <t>ruins_trace</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -5335,7 +5333,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>지역 흔적 아이템명</t>
+          <t>지역 흔적 아이템 ID</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5362,30 +5360,32 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>hidden_stage_required_amount</t>
-        </is>
-      </c>
-      <c r="C71" t="n">
-        <v>20</v>
+          <t>trace_name</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>화염의 잔재</t>
+        </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Hidden Stage 입장 흔적 수</t>
+          <t>지역 흔적 아이템명</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>입장 난이도↑</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>입장 난이도↓</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -5402,32 +5402,30 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>next_region_id</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>dark_swamp</t>
-        </is>
+          <t>hidden_stage_required_amount</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>20</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>다음 지역 ID</t>
+          <t>Hidden Stage 입장 흔적 수</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>입장 난이도↑</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>입장 난이도↓</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -5444,30 +5442,32 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>next_region_unlock_level</t>
-        </is>
-      </c>
-      <c r="C73" t="n">
-        <v>80</v>
+          <t>next_region_id</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>dark_swamp</t>
+        </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>다음 지역 해금 레벨</t>
+          <t>다음 지역 ID</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>해금 지연</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>해금 빨라짐</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -5484,30 +5484,30 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>weight_material</t>
+          <t>next_region_unlock_level</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>level</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>탐색률 재료 기여</t>
+          <t>다음 지역 해금 레벨</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>비중↑</t>
+          <t>해금 지연</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>비중↓</t>
+          <t>해금 빨라짐</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>weight_spirit</t>
+          <t>weight_material</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -5537,7 +5537,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>탐색률 정령 기여</t>
+          <t>탐색률 재료 기여</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>weight_regional</t>
+          <t>weight_spirit</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>탐색률 지역 기여</t>
+          <t>탐색률 정령 기여</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -5604,11 +5604,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>weight_treasure</t>
+          <t>weight_regional</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -5617,7 +5617,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>탐색률 보물 기여</t>
+          <t>탐색률 지역 기여</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -5644,30 +5644,30 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>total_material_discovery</t>
+          <t>weight_treasure</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>weight</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>재료 발견 총량</t>
+          <t>탐색률 보물 기여</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>완료 난이도↑</t>
+          <t>비중↑</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>완료 난이도↓</t>
+          <t>비중↓</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -5684,11 +5684,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>total_spirit_discovery</t>
+          <t>total_material_discovery</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>정령 발견 총량</t>
+          <t>재료 발견 총량</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -5724,11 +5724,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>total_regional_discovery</t>
+          <t>total_spirit_discovery</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -5737,7 +5737,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>지역 발견 총량</t>
+          <t>정령 발견 총량</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -5764,11 +5764,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>total_treasure_discovery</t>
+          <t>total_regional_discovery</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -5777,7 +5777,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>보물 발견 총량</t>
+          <t>지역 발견 총량</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -5799,37 +5799,35 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Map5</t>
+          <t>Map4</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>region_id</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>dark_swamp</t>
-        </is>
+          <t>total_treasure_discovery</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>1</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>현재 적용 지역 ID</t>
+          <t>보물 발견 총량</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>완료 난이도↑</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>완료 난이도↓</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -5846,12 +5844,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>region_name</t>
+          <t>region_id</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>어둠의 습지</t>
+          <t>dark_swamp</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5861,7 +5859,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>현재 적용 지역명</t>
+          <t>현재 적용 지역 ID</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -5888,30 +5886,32 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>unlock_level</t>
-        </is>
-      </c>
-      <c r="C84" t="n">
-        <v>80</v>
+          <t>region_name</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>어둠의 습지</t>
+        </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>입장 레벨</t>
+          <t>현재 적용 지역명</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>해금 지연</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>해금 빨라짐</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -5928,7 +5928,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>recommended_level</t>
+          <t>unlock_level</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -5941,17 +5941,17 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>권장 레벨</t>
+          <t>입장 레벨</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>권장치 상승</t>
+          <t>해금 지연</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>권장치 하락</t>
+          <t>해금 빨라짐</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -5968,30 +5968,30 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>mana_cost</t>
+          <t>recommended_level</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>mana</t>
+          <t>level</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>탐사 1회 입장 소모 마나</t>
+          <t>권장 레벨</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>비용 증가</t>
+          <t>권장치 상승</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>비용 감소</t>
+          <t>권장치 하락</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -6008,30 +6008,30 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>explore_steps</t>
+          <t>mana_cost</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>mana</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>탐색 행동 횟수</t>
+          <t>탐사 1회 입장 소모 마나</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>탐험 길어짐</t>
+          <t>비용 증가</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>탐험 짧아짐</t>
+          <t>비용 감소</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -6048,32 +6048,30 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>trace_item_id</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>final_trace</t>
-        </is>
+          <t>explore_steps</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>10</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>지역 흔적 아이템 ID</t>
+          <t>탐색 행동 횟수</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>탐험 길어짐</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>탐험 짧아짐</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -6090,12 +6088,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>trace_name</t>
+          <t>trace_item_id</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>어둠의 흔적</t>
+          <t>final_trace</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -6105,7 +6103,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>지역 흔적 아이템명</t>
+          <t>지역 흔적 아이템 ID</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6132,30 +6130,32 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>hidden_stage_required_amount</t>
-        </is>
-      </c>
-      <c r="C90" t="n">
-        <v>20</v>
+          <t>trace_name</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>어둠의 흔적</t>
+        </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Hidden Stage 입장 흔적 수</t>
+          <t>지역 흔적 아이템명</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>입장 난이도↑</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>입장 난이도↓</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -6172,27 +6172,30 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>next_region_id</t>
-        </is>
+          <t>hidden_stage_required_amount</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>20</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>다음 지역 ID</t>
+          <t>Hidden Stage 입장 흔적 수</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>입장 난이도↑</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>입장 난이도↓</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -6209,30 +6212,27 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>next_region_unlock_level</t>
-        </is>
-      </c>
-      <c r="C92" t="n">
-        <v>0</v>
+          <t>next_region_id</t>
+        </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>다음 지역 해금 레벨</t>
+          <t>다음 지역 ID</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>해금 지연</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>해금 빨라짐</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -6249,30 +6249,30 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>weight_material</t>
+          <t>next_region_unlock_level</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>level</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>탐색률 재료 기여</t>
+          <t>다음 지역 해금 레벨</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>비중↑</t>
+          <t>해금 지연</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>비중↓</t>
+          <t>해금 빨라짐</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -6289,7 +6289,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>weight_spirit</t>
+          <t>weight_material</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>탐색률 정령 기여</t>
+          <t>탐색률 재료 기여</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -6329,7 +6329,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>weight_regional</t>
+          <t>weight_spirit</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>탐색률 지역 기여</t>
+          <t>탐색률 정령 기여</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -6369,11 +6369,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>weight_treasure</t>
+          <t>weight_regional</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>탐색률 보물 기여</t>
+          <t>탐색률 지역 기여</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -6409,30 +6409,30 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>total_material_discovery</t>
+          <t>weight_treasure</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>weight</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>재료 발견 총량</t>
+          <t>탐색률 보물 기여</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>완료 난이도↑</t>
+          <t>비중↑</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>완료 난이도↓</t>
+          <t>비중↓</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -6449,11 +6449,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>total_spirit_discovery</t>
+          <t>total_material_discovery</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>정령 발견 총량</t>
+          <t>재료 발견 총량</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -6489,11 +6489,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>total_regional_discovery</t>
+          <t>total_spirit_discovery</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -6502,7 +6502,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>지역 발견 총량</t>
+          <t>정령 발견 총량</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -6529,33 +6529,73 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
+          <t>total_regional_discovery</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>4</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>지역 발견 총량</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>완료 난이도↑</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>완료 난이도↓</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>src/data/regions.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Map5</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
           <t>total_treasure_discovery</t>
         </is>
       </c>
-      <c r="C100" t="n">
-        <v>1</v>
-      </c>
-      <c r="D100" t="inlineStr">
+      <c r="C101" t="n">
+        <v>1</v>
+      </c>
+      <c r="D101" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
+      <c r="E101" t="inlineStr">
         <is>
           <t>보물 발견 총량</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr">
+      <c r="F101" t="inlineStr">
         <is>
           <t>완료 난이도↑</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr">
+      <c r="G101" t="inlineStr">
         <is>
           <t>완료 난이도↓</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr">
+      <c r="H101" t="inlineStr">
         <is>
           <t>src/data/regions.ts</t>
         </is>

</xml_diff>